<commit_message>
feat: peer assesment completed
</commit_message>
<xml_diff>
--- a/My_Professional_Reviews/UAS-5_Skor_Peer.xlsx
+++ b/My_Professional_Reviews/UAS-5_Skor_Peer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raihaan\all-about-me\My_Professional_Reviews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30383C08-305F-44B3-A119-15B4064FF751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C6E4F1-B304-4262-BA05-E046F9B43637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
   </bookViews>
   <sheets>
     <sheet name="UAS_1_My_Concepts" sheetId="2" r:id="rId1"/>
@@ -132,9 +132,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -212,18 +219,19 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,7 +651,22 @@
       <c r="B3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="C3" s="2">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>4</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="7">
+        <f>AVERAGE(C3:F3)</f>
+        <v>4.5</v>
+      </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="V3" s="4"/>
@@ -672,7 +695,7 @@
         <v>5</v>
       </c>
       <c r="G4" s="4">
-        <f t="shared" ref="G3:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
+        <f>IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
         <v>4.75</v>
       </c>
       <c r="L4" s="4"/>
@@ -690,7 +713,22 @@
       <c r="B5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="4"/>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f>AVERAGE(C5:F5)</f>
+        <v>5</v>
+      </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="V5" s="4"/>
@@ -701,7 +739,7 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G6" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G4:G66" si="0">IF(COUNT(C6:F6)=0,"",AVERAGE(C6:F6))</f>
         <v/>
       </c>
       <c r="L6" s="4"/>
@@ -1817,7 +1855,22 @@
       <c r="B3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <f>AVERAGE(C3:F3)</f>
+        <v>5</v>
+      </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="V3" s="4"/>
@@ -1846,7 +1899,7 @@
         <v>5</v>
       </c>
       <c r="G4" s="4">
-        <f t="shared" ref="G3:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
+        <f t="shared" ref="G4:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
         <v>4.75</v>
       </c>
       <c r="L4" s="4"/>
@@ -1864,7 +1917,22 @@
       <c r="B5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="4"/>
+      <c r="C5" s="2">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f>AVERAGE(C5:F5)</f>
+        <v>4.5</v>
+      </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="V5" s="4"/>
@@ -2991,7 +3059,22 @@
       <c r="B3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="C3" s="2">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <f>AVERAGE(C3:F3)</f>
+        <v>4.75</v>
+      </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="V3" s="4"/>
@@ -3020,7 +3103,7 @@
         <v>4</v>
       </c>
       <c r="G4" s="4">
-        <f t="shared" ref="G3:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
+        <f t="shared" ref="G4:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
         <v>4.5</v>
       </c>
       <c r="L4" s="4"/>
@@ -3038,7 +3121,22 @@
       <c r="B5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="4"/>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f>AVERAGE(C5:F5)</f>
+        <v>4.75</v>
+      </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="V5" s="4"/>
@@ -4165,7 +4263,22 @@
       <c r="B3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
+        <f>AVERAGE(C3:F3)</f>
+        <v>4.75</v>
+      </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="V3" s="4"/>
@@ -4194,7 +4307,7 @@
         <v>5</v>
       </c>
       <c r="G4" s="4">
-        <f t="shared" ref="G3:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
+        <f t="shared" ref="G4:G66" si="0">IF(COUNT(C4:F4)=0,"",AVERAGE(C4:F4))</f>
         <v>4.75</v>
       </c>
       <c r="L4" s="4"/>
@@ -4212,7 +4325,22 @@
       <c r="B5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="4"/>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f>AVERAGE(C5:F5)</f>
+        <v>4.75</v>
+      </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="V5" s="4"/>

</xml_diff>